<commit_message>
chore: weekly update 20260623
</commit_message>
<xml_diff>
--- a/long-short strategy/000832_CSI_close_price.xlsx
+++ b/long-short strategy/000832_CSI_close_price.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2293"/>
+  <dimension ref="A1:B2298"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18786,6 +18786,46 @@
         <v>497.3402</v>
       </c>
     </row>
+    <row r="2294">
+      <c r="A2294" s="1" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B2294" t="n">
+        <v>498.7353</v>
+      </c>
+    </row>
+    <row r="2295">
+      <c r="A2295" s="1" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B2295" t="n">
+        <v>503.3438</v>
+      </c>
+    </row>
+    <row r="2296">
+      <c r="A2296" s="1" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B2296" t="n">
+        <v>511.0471</v>
+      </c>
+    </row>
+    <row r="2297">
+      <c r="A2297" s="1" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B2297" t="n">
+        <v>513.6308</v>
+      </c>
+    </row>
+    <row r="2298">
+      <c r="A2298" s="1" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B2298" t="n">
+        <v>512.1285</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: weekly update 20260710
</commit_message>
<xml_diff>
--- a/long-short strategy/000832_CSI_close_price.xlsx
+++ b/long-short strategy/000832_CSI_close_price.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2309"/>
+  <dimension ref="A1:B2314"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18914,6 +18914,46 @@
         <v>506.9109</v>
       </c>
     </row>
+    <row r="2310">
+      <c r="A2310" s="1" t="n">
+        <v>46209</v>
+      </c>
+      <c r="B2310" t="n">
+        <v>507.1223</v>
+      </c>
+    </row>
+    <row r="2311">
+      <c r="A2311" s="1" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B2311" t="n">
+        <v>502.2414</v>
+      </c>
+    </row>
+    <row r="2312">
+      <c r="A2312" s="1" t="n">
+        <v>46211</v>
+      </c>
+      <c r="B2312" t="n">
+        <v>500.4418</v>
+      </c>
+    </row>
+    <row r="2313">
+      <c r="A2313" s="1" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B2313" t="n">
+        <v>503.2105</v>
+      </c>
+    </row>
+    <row r="2314">
+      <c r="A2314" s="1" t="n">
+        <v>46213</v>
+      </c>
+      <c r="B2314" t="n">
+        <v>500.5492</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>